<commit_message>
UAR simulation: hard-mode data, request and exception logs, README source fixes
Adds access-requests.csv and exceptions-register.csv, richer synthetic credential history, and a README section on which source is authoritative (synthetic credential report for credential activity and age, live IAM for structure and entitlements). Status line now reflects the deployed tag live-2026-10-14-2 with the hard-mode update pending deployment. Infrastructure and the generator live only in the 340collective-website repo.
</commit_message>
<xml_diff>
--- a/08-access-reviews/uar-simulation/data/uar-worksheet.xlsx
+++ b/08-access-reviews/uar-simulation/data/uar-worksheet.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A34"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -512,7 +512,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Access Level: the highest level implied by those policies (Admin, PowerUser, Write, Read, None).</t>
+          <t>Access Level: the highest level implied by those policies (Admin, PowerUser, Write, Read, None). It is derived from policy names, so treat it as a starting point, not evidence; read the policy documents.</t>
         </is>
       </c>
     </row>
@@ -637,22 +637,46 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Live IAM (path /uar-sim/): groups, attached and inline policies, and tags for every synthetic user.</t>
+          <t>access-requests.csv: access request and approval log. Keys: requester and approver (HR employee_id), beneficiary (Identity).</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>exceptions-register.csv: approved exceptions to the access standard. Keys: identity (Identity), approver (HR employee_id).</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
+          <t>Live IAM (path /uar-sim/): users, groups, attached and inline policies, policy documents, roles, trust policies, and tags.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Which source is authoritative: the synthetic aws-credential-report.csv for passwords, MFA, and access key age and use; live IAM for structure and entitlements (users, groups, policies, roles, trust, tags).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
           <t>Names are not a reliable join key. Join on employee ID, IAM user name, or email.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Log every Reduce or Remove decision on the Remediation Log sheet with a target date.</t>
         </is>
@@ -2167,7 +2191,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>Groups: uar-sim-Sales-CRM, uar-sim-Data-Analysts</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -2872,7 +2896,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>No activity recorded</t>
         </is>
       </c>
       <c r="G60" t="inlineStr"/>
@@ -3069,7 +3093,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>elizabeth.banerjee@example.com</t>
+          <t>eli.sterling@example.com</t>
         </is>
       </c>
       <c r="B66" t="inlineStr"/>
@@ -3098,14 +3122,10 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>emendoza</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>E10131</t>
-        </is>
-      </c>
+          <t>elizabeth.banerjee@example.com</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>person</t>
@@ -3113,19 +3133,15 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Change-Approvers, uar-sim-ReadOnly</t>
+          <t>No AWS account</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Write</t>
-        </is>
-      </c>
-      <c r="F67" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
       <c r="H67" t="inlineStr"/>
       <c r="I67" t="inlineStr"/>
@@ -3135,12 +3151,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>enwosu</t>
+          <t>emendoza</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>E10168</t>
+          <t>E10131</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3150,17 +3166,17 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Marketing, uar-sim-Admins</t>
+          <t>Groups: uar-sim-Change-Approvers, uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G68" t="inlineStr"/>
@@ -3172,12 +3188,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>eramirez</t>
+          <t>enwosu</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>E10025</t>
+          <t>E10168</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3187,17 +3203,17 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>Groups: uar-sim-Marketing, uar-sim-Admins</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="G69" t="inlineStr"/>
@@ -3209,12 +3225,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>esterling</t>
+          <t>eramirez</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>E10203</t>
+          <t>E10025</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3224,7 +3240,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -3234,7 +3250,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="G70" t="inlineStr"/>
@@ -3246,10 +3262,14 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>esther.conway@example.com</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
+          <t>esterling</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>E10203</t>
+        </is>
+      </c>
       <c r="C71" t="inlineStr">
         <is>
           <t>person</t>
@@ -3257,15 +3277,19 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>No AWS account</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F71" t="inlineStr"/>
+          <t>Write</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr"/>
@@ -3275,14 +3299,10 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>evelasco</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>E10083</t>
-        </is>
-      </c>
+          <t>esther.conway@example.com</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>person</t>
@@ -3290,19 +3310,15 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>No AWS account</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Write</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>2026-05-04</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
@@ -3312,12 +3328,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>fdorsey</t>
+          <t>evelasco</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>E10202</t>
+          <t>E10083</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3337,7 +3353,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="G73" t="inlineStr"/>
@@ -3349,12 +3365,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>frosales</t>
+          <t>fdorsey</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>E10170</t>
+          <t>E10202</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3364,7 +3380,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Finance-Payments-Create</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -3374,7 +3390,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="G74" t="inlineStr"/>
@@ -3386,12 +3402,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>fyamamoto</t>
+          <t>frosales</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>E10050</t>
+          <t>E10170</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3411,7 +3427,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="G75" t="inlineStr"/>
@@ -3423,12 +3439,12 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>gcarver</t>
+          <t>fyamamoto</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>E10100</t>
+          <t>E10050</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3438,7 +3454,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Finance-Payments-Create</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -3448,7 +3464,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G76" t="inlineStr"/>
@@ -3460,12 +3476,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>gfoley</t>
+          <t>gcarver</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>E10107</t>
+          <t>E10100</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3475,7 +3491,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM, uar-sim-Marketing; Inline: uar-sim-campaign-tools</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -3485,7 +3501,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="G77" t="inlineStr"/>
@@ -3497,12 +3513,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>gnovak</t>
+          <t>gfoley</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>E10075</t>
+          <t>E10107</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -3512,17 +3528,17 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Sales-CRM, uar-sim-Marketing; Inline: uar-sim-campaign-tools</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="G78" t="inlineStr"/>
@@ -3534,12 +3550,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>gsullivan</t>
+          <t>gnovak</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>E10004</t>
+          <t>E10075</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -3559,7 +3575,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="G79" t="inlineStr"/>
@@ -3571,12 +3587,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>hcarver</t>
+          <t>gsullivan</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>E10128</t>
+          <t>E10004</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -3586,17 +3602,17 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Read</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="G80" t="inlineStr"/>
@@ -3608,10 +3624,14 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>hector.langley@example.com</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr"/>
+          <t>hcarver</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>E10128</t>
+        </is>
+      </c>
       <c r="C81" t="inlineStr">
         <is>
           <t>person</t>
@@ -3619,15 +3639,19 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>No AWS account</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr"/>
+          <t>Write</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
       <c r="G81" t="inlineStr"/>
       <c r="H81" t="inlineStr"/>
       <c r="I81" t="inlineStr"/>
@@ -3637,14 +3661,10 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>hgentry</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>E10198</t>
-        </is>
-      </c>
+          <t>hector.langley@example.com</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
           <t>person</t>
@@ -3652,19 +3672,15 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-HR-Records</t>
+          <t>No AWS account</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Write</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr"/>
@@ -3674,12 +3690,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>hmadsen</t>
+          <t>hgentry</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>E10020</t>
+          <t>E10198</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -3689,7 +3705,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Finance-Payments-Approve</t>
+          <t>Groups: uar-sim-HR-Records</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3699,7 +3715,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G83" t="inlineStr"/>
@@ -3711,12 +3727,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>hsolis</t>
+          <t>hmadsen</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>C20013</t>
+          <t>E10020</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -3726,7 +3742,7 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Contractors</t>
+          <t>Groups: uar-sim-Finance-Payments-Approve</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3736,7 +3752,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G84" t="inlineStr"/>
@@ -3748,12 +3764,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>hvasquez</t>
+          <t>hsolis</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>E10079</t>
+          <t>C20013</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -3763,7 +3779,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Data-Analysts</t>
+          <t>Groups: uar-sim-Contractors</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -3773,7 +3789,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="G85" t="inlineStr"/>
@@ -3785,12 +3801,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>hwaller</t>
+          <t>hvasquez</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>E10074</t>
+          <t>E10079</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -3800,17 +3816,17 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-PowerUsers</t>
+          <t>Groups: uar-sim-Data-Analysts</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>PowerUser</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="G86" t="inlineStr"/>
@@ -3822,12 +3838,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>hwhitfield</t>
+          <t>hwaller</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>E10163</t>
+          <t>E10074</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -3837,17 +3853,17 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>Groups: uar-sim-PowerUsers, uar-sim-Admins</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="G87" t="inlineStr"/>
@@ -3859,12 +3875,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>hwhitfield2</t>
+          <t>hwhitfield</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>E10186</t>
+          <t>E10163</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -3874,7 +3890,7 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Engineering-Deploy, uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3884,7 +3900,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="G88" t="inlineStr"/>
@@ -3896,12 +3912,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>hzeller</t>
+          <t>hwhitfield2</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>E10052</t>
+          <t>E10186</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -3911,7 +3927,7 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Engineering-Deploy, uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Engineering-Deploy, uar-sim-ReadOnly, uar-sim-Data-Analysts</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3921,7 +3937,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="G89" t="inlineStr"/>
@@ -3933,12 +3949,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>iandersen</t>
+          <t>hzeller</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>E10026</t>
+          <t>E10052</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -3948,7 +3964,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>Groups: uar-sim-Engineering-Deploy, uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -3958,7 +3974,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="G90" t="inlineStr"/>
@@ -3970,12 +3986,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ibishop</t>
+          <t>iandersen</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>E10073</t>
+          <t>E10026</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -3985,17 +4001,17 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="G91" t="inlineStr"/>
@@ -4007,12 +4023,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>icrane</t>
+          <t>ibishop</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>E10166</t>
+          <t>E10073</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4022,17 +4038,17 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly; Policies: uar-sim-ops-break-glass</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Read</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="G92" t="inlineStr"/>
@@ -4044,12 +4060,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>ieaston</t>
+          <t>icrane</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>E10174</t>
+          <t>E10166</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4059,7 +4075,7 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM; Policies: AdministratorAccess</t>
+          <t>Groups: uar-sim-ReadOnly; Policies: uar-sim-ops-break-glass</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -4069,7 +4085,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="G93" t="inlineStr"/>
@@ -4081,12 +4097,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>iholloway</t>
+          <t>ieaston</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>E10184</t>
+          <t>E10174</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4096,17 +4112,17 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Sales-CRM; Policies: AdministratorAccess</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="G94" t="inlineStr"/>
@@ -4118,12 +4134,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>ihuang</t>
+          <t>iholloway</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>E10161</t>
+          <t>E10184</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4133,7 +4149,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-HR-Records</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -4143,7 +4159,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="G95" t="inlineStr"/>
@@ -4155,12 +4171,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ilozano</t>
+          <t>ihuang</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>E10033</t>
+          <t>E10161</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4170,7 +4186,7 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets, uar-sim-Data-Analysts</t>
+          <t>Groups: uar-sim-HR-Records</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
@@ -4180,7 +4196,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G96" t="inlineStr"/>
@@ -4192,12 +4208,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>imontague</t>
+          <t>ilozano</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>E10042</t>
+          <t>E10033</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4207,17 +4223,17 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Creative-Assets, uar-sim-Data-Analysts</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="G97" t="inlineStr"/>
@@ -4229,10 +4245,14 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>isabel.oyelaran@example.com</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr"/>
+          <t>imontague</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>E10042</t>
+        </is>
+      </c>
       <c r="C98" t="inlineStr">
         <is>
           <t>person</t>
@@ -4240,15 +4260,19 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>No AWS account</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr"/>
+          <t>Read</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
       <c r="G98" t="inlineStr"/>
       <c r="H98" t="inlineStr"/>
       <c r="I98" t="inlineStr"/>
@@ -4258,14 +4282,10 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>iserrano</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>E10109</t>
-        </is>
-      </c>
+          <t>isabel.oyelaran@example.com</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
           <t>person</t>
@@ -4273,19 +4293,15 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>No AWS account</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Write</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr"/>
       <c r="H99" t="inlineStr"/>
       <c r="I99" t="inlineStr"/>
@@ -4295,12 +4311,12 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>iunderwood</t>
+          <t>iserrano</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>E10205</t>
+          <t>E10109</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -4310,7 +4326,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -4320,7 +4336,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="G100" t="inlineStr"/>
@@ -4332,12 +4348,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>jadeyemi</t>
+          <t>iunderwood</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>E10055</t>
+          <t>E10205</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -4347,17 +4363,17 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>No activity recorded</t>
         </is>
       </c>
       <c r="G101" t="inlineStr"/>
@@ -4369,12 +4385,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>jduarte</t>
+          <t>jadeyemi</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>E10063</t>
+          <t>E10055</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -4384,17 +4400,17 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Read</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="G102" t="inlineStr"/>
@@ -4406,12 +4422,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>jfoley</t>
+          <t>jduarte</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>E10028</t>
+          <t>E10063</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -4421,7 +4437,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -4431,7 +4447,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
@@ -4443,12 +4459,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>jhuang</t>
+          <t>jfoley</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>E10036</t>
+          <t>E10028</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -4458,7 +4474,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Finance-Payments-Approve, uar-sim-Finance-Payments-Create</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -4468,7 +4484,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
@@ -4480,12 +4496,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>jmadsen</t>
+          <t>jhuang</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>E10048</t>
+          <t>E10036</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -4495,7 +4511,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Finance-Payments-Approve, uar-sim-Finance-Payments-Create</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -4505,7 +4521,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="G105" t="inlineStr"/>
@@ -4517,12 +4533,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>jmarsh</t>
+          <t>jmadsen</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>E10001</t>
+          <t>E10048</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4532,17 +4548,17 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="G106" t="inlineStr"/>
@@ -4554,12 +4570,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>jmercer</t>
+          <t>jmarsh</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>E10199</t>
+          <t>E10001</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -4579,7 +4595,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="G107" t="inlineStr"/>
@@ -4591,12 +4607,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>jmolina</t>
+          <t>jmercer</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>E10121</t>
+          <t>E10199</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -4606,17 +4622,17 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Read</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G108" t="inlineStr"/>
@@ -4628,12 +4644,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>jthornton</t>
+          <t>jmolina</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>E10178</t>
+          <t>E10121</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -4643,7 +4659,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -4653,7 +4669,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="G109" t="inlineStr"/>
@@ -4665,12 +4681,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>jyamamoto</t>
+          <t>jthornton</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>E10143</t>
+          <t>E10178</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -4680,7 +4696,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -4690,7 +4706,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="G110" t="inlineStr"/>
@@ -4702,12 +4718,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>kemerson</t>
+          <t>jyamamoto</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>E10193</t>
+          <t>E10143</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -4727,7 +4743,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G111" t="inlineStr"/>
@@ -4739,12 +4755,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>kfontaine</t>
+          <t>kemerson</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>E10185</t>
+          <t>E10193</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -4754,7 +4770,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
@@ -4764,7 +4780,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="G112" t="inlineStr"/>
@@ -4776,12 +4792,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>kgallagher</t>
+          <t>kfontaine</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>E10066</t>
+          <t>E10185</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -4791,17 +4807,17 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Admins</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>Admin</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="G113" t="inlineStr"/>
@@ -4813,12 +4829,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>khamada</t>
+          <t>kgallagher</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>E10076</t>
+          <t>E10066</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4828,17 +4844,17 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets, uar-sim-Marketing</t>
+          <t>Groups: uar-sim-Admins</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Admin</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="G114" t="inlineStr"/>
@@ -4850,12 +4866,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>kiverson</t>
+          <t>khamada</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>E10006</t>
+          <t>E10076</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -4865,17 +4881,17 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Creative-Assets, uar-sim-Marketing</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="G115" t="inlineStr"/>
@@ -4887,12 +4903,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>krivera</t>
+          <t>kiverson</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>E10171</t>
+          <t>E10006</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -4902,17 +4918,17 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Data-Analysts</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Read</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="G116" t="inlineStr"/>
@@ -4924,12 +4940,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ktanaka</t>
+          <t>krivera</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>E10155</t>
+          <t>E10171</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -4939,7 +4955,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Data-Analysts, uar-sim-Engineering-Deploy</t>
+          <t>Groups: uar-sim-Data-Analysts</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -4949,7 +4965,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G117" t="inlineStr"/>
@@ -4961,12 +4977,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>kunderwood</t>
+          <t>ktanaka</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>E10093</t>
+          <t>E10155</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -4976,17 +4992,17 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Data-Analysts, uar-sim-Engineering-Deploy</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="G118" t="inlineStr"/>
@@ -4998,12 +5014,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>kwhitfield</t>
+          <t>kunderwood</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>E10158</t>
+          <t>E10093</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -5023,7 +5039,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="G119" t="inlineStr"/>
@@ -5035,12 +5051,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>kzeller</t>
+          <t>kwhitfield</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>E10097</t>
+          <t>E10158</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -5060,7 +5076,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G120" t="inlineStr"/>
@@ -5072,12 +5088,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>lacosta</t>
+          <t>kzeller</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>E10196</t>
+          <t>E10097</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -5087,17 +5103,17 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Engineering-Deploy, uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Read</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="G121" t="inlineStr"/>
@@ -5109,12 +5125,12 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>landersen</t>
+          <t>lacosta</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>E10018</t>
+          <t>E10196</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -5124,7 +5140,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Engineering-Deploy, uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -5134,7 +5150,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="G122" t="inlineStr"/>
@@ -5146,12 +5162,12 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>lbarrett</t>
+          <t>landersen</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>C20006</t>
+          <t>E10018</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -5161,7 +5177,7 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Contractors, uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -5171,7 +5187,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="G123" t="inlineStr"/>
@@ -5183,12 +5199,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>lbolton</t>
+          <t>lbarrett</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>E10096</t>
+          <t>C20006</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -5198,7 +5214,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Finance-Payments-Approve</t>
+          <t>Groups: uar-sim-Contractors, uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5208,7 +5224,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>2025-08-16</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="G124" t="inlineStr"/>
@@ -5220,12 +5236,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>lcollier</t>
+          <t>lbolton</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>E10009</t>
+          <t>E10096</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -5235,7 +5251,7 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Finance-Payments-Approve</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -5245,7 +5261,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2025-08-16</t>
         </is>
       </c>
       <c r="G125" t="inlineStr"/>
@@ -5257,12 +5273,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>lcrane</t>
+          <t>lcollier</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>C20017</t>
+          <t>E10009</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -5272,7 +5288,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Contractors</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -5282,7 +5298,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>2026-09-25</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="G126" t="inlineStr"/>
@@ -5294,12 +5310,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ldempsey</t>
+          <t>lcrane</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>E10049</t>
+          <t>C20017</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -5309,17 +5325,17 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Contractors</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="G127" t="inlineStr"/>
@@ -5331,12 +5347,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>lholloway</t>
+          <t>ldempsey</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>C20023</t>
+          <t>E10049</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -5346,17 +5362,17 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Contractors</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Read</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="G128" t="inlineStr"/>
@@ -5368,12 +5384,12 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>lmercer</t>
+          <t>lholloway</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>C20018</t>
+          <t>C20023</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -5383,7 +5399,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Contractors, uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Contractors</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -5393,7 +5409,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="G129" t="inlineStr"/>
@@ -5405,12 +5421,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>lrosales</t>
+          <t>lmercer</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>E10059</t>
+          <t>C20018</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -5420,7 +5436,7 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Change-Approvers, uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-Contractors, uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
@@ -5430,7 +5446,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="G130" t="inlineStr"/>
@@ -5442,12 +5458,12 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>lvelasco</t>
+          <t>lrosales</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>C20007</t>
+          <t>E10059</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -5457,7 +5473,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Contractors</t>
+          <t>Groups: uar-sim-Change-Approvers, uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -5467,7 +5483,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="G131" t="inlineStr"/>
@@ -5479,10 +5495,14 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>marcus.abernathy@example.com</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr"/>
+          <t>lvelasco</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>C20007</t>
+        </is>
+      </c>
       <c r="C132" t="inlineStr">
         <is>
           <t>person</t>
@@ -5490,15 +5510,19 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>No AWS account</t>
+          <t>Groups: uar-sim-Contractors</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr"/>
+          <t>Write</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
       <c r="G132" t="inlineStr"/>
       <c r="H132" t="inlineStr"/>
       <c r="I132" t="inlineStr"/>
@@ -5508,7 +5532,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>marketing-team</t>
+          <t>marcus.abernathy@example.com</t>
         </is>
       </c>
       <c r="B133" t="inlineStr"/>
@@ -5519,19 +5543,15 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Marketing</t>
+          <t>No AWS account</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Write</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>2026-08-27</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr"/>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="inlineStr"/>
       <c r="I133" t="inlineStr"/>
@@ -5541,14 +5561,10 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>mbowers</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>E10061</t>
-        </is>
-      </c>
+          <t>marketing-team</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
           <t>person</t>
@@ -5556,7 +5572,7 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Marketing</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
@@ -5566,7 +5582,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="G134" t="inlineStr"/>
@@ -5578,12 +5594,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>mbrennan</t>
+          <t>mbowers</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>E10151</t>
+          <t>E10061</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -5593,7 +5609,7 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Marketing</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
@@ -5603,7 +5619,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>2026-01-03</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="G135" t="inlineStr"/>
@@ -5615,12 +5631,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>mcalloway</t>
+          <t>mbrennan</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>C20012</t>
+          <t>E10151</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -5630,17 +5646,17 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Contractors, uar-sim-Creative-Assets, uar-sim-PowerUsers</t>
+          <t>Groups: uar-sim-Marketing</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>PowerUser</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="G136" t="inlineStr"/>
@@ -5652,12 +5668,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>mcalloway2</t>
+          <t>mcalloway</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>E10123</t>
+          <t>C20012</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -5667,17 +5683,17 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-HR-Records</t>
+          <t>Groups: uar-sim-Contractors, uar-sim-Creative-Assets, uar-sim-PowerUsers</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>PowerUser</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="G137" t="inlineStr"/>
@@ -5689,12 +5705,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>mcampos</t>
+          <t>mcalloway2</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>E10197</t>
+          <t>E10123</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -5704,17 +5720,17 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-HR-Records</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>Write</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G138" t="inlineStr"/>
@@ -5726,12 +5742,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>measton</t>
+          <t>mcampos</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>E10120</t>
+          <t>E10197</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -5741,17 +5757,17 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-ReadOnly</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Write</t>
+          <t>Read</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G139" t="inlineStr"/>
@@ -5763,10 +5779,14 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>megan.holloway@example.com</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr"/>
+          <t>measton</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>E10120</t>
+        </is>
+      </c>
       <c r="C140" t="inlineStr">
         <is>
           <t>person</t>
@@ -5774,15 +5794,19 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>No AWS account</t>
+          <t>Groups: uar-sim-Creative-Assets</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F140" t="inlineStr"/>
+          <t>Write</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="G140" t="inlineStr"/>
       <c r="H140" t="inlineStr"/>
       <c r="I140" t="inlineStr"/>
@@ -5792,14 +5816,10 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>mgarrison</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>E10011</t>
-        </is>
-      </c>
+          <t>megan.holloway@example.com</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr">
         <is>
           <t>person</t>
@@ -5807,19 +5827,15 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>No AWS account</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Write</t>
-        </is>
-      </c>
-      <c r="F141" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr"/>
       <c r="G141" t="inlineStr"/>
       <c r="H141" t="inlineStr"/>
       <c r="I141" t="inlineStr"/>
@@ -5829,12 +5845,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>mhalloway</t>
+          <t>mgarrison</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>E10139</t>
+          <t>E10011</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -5854,7 +5870,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G142" t="inlineStr"/>
@@ -5866,12 +5882,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>mibarra</t>
+          <t>mhalloway</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>E10119</t>
+          <t>E10139</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -5881,7 +5897,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Marketing</t>
+          <t>Groups: uar-sim-Sales-CRM</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -5891,7 +5907,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="G143" t="inlineStr"/>
@@ -5903,10 +5919,14 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>mila.solis@example.com</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr"/>
+          <t>mibarra</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>E10119</t>
+        </is>
+      </c>
       <c r="C144" t="inlineStr">
         <is>
           <t>person</t>
@@ -5914,15 +5934,19 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>No AWS account</t>
+          <t>Groups: uar-sim-Marketing</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="F144" t="inlineStr"/>
+          <t>Write</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="G144" t="inlineStr"/>
       <c r="H144" t="inlineStr"/>
       <c r="I144" t="inlineStr"/>
@@ -6031,7 +6055,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="G147" t="inlineStr"/>
@@ -6216,7 +6240,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="G152" t="inlineStr"/>
@@ -6354,7 +6378,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Creative-Assets</t>
+          <t>Groups: uar-sim-Creative-Assets, uar-sim-Marketing</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -6922,7 +6946,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-ReadOnly, uar-sim-Reporting</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
@@ -8696,7 +8720,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-Sales-CRM</t>
+          <t>Groups: uar-sim-Sales-CRM, uar-sim-Data-Analysts</t>
         </is>
       </c>
       <c r="E222" t="inlineStr">
@@ -9056,7 +9080,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="G232" t="inlineStr"/>
@@ -9231,12 +9255,12 @@
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Groups: uar-sim-ReadOnly</t>
+          <t>Groups: uar-sim-ReadOnly, uar-sim-PowerUsers</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Read</t>
+          <t>PowerUser</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">

</xml_diff>